<commit_message>
Cosine lr scheduling enabled
</commit_message>
<xml_diff>
--- a/project/network_performance.xlsx
+++ b/project/network_performance.xlsx
@@ -52,7 +52,7 @@
     <t xml:space="preserve">test set</t>
   </si>
   <si>
-    <t xml:space="preserve">NEMA</t>
+    <t xml:space="preserve">NEMA (center slices)</t>
   </si>
   <si>
     <t xml:space="preserve">Notes</t>
@@ -185,7 +185,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -194,20 +194,28 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -411,55 +419,56 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="20.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="18.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="12.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="9.1"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="5"/>
+    </row>
+    <row r="2" customFormat="false" ht="35.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
       <c r="E2" s="4"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="5" t="s">
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="K2" s="5" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Moved tuned config dicts into project directory
</commit_message>
<xml_diff>
--- a/project/network_performance.xlsx
+++ b/project/network_performance.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="63">
   <si>
     <t xml:space="preserve">Recon Type</t>
   </si>
@@ -46,6 +46,12 @@
     <t xml:space="preserve">SSIM</t>
   </si>
   <si>
+    <t xml:space="preserve">MSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lr min factor</t>
   </si>
   <si>
@@ -67,6 +73,9 @@
     <t xml:space="preserve">NEMA CRC (17 mm)</t>
   </si>
   <si>
+    <t xml:space="preserve">NEMA</t>
+  </si>
+  <si>
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
@@ -79,6 +88,12 @@
     <t xml:space="preserve">0.916738 +/- 0.042070</t>
   </si>
   <si>
+    <t xml:space="preserve">39.014 +/- 59.210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31.750 +/- 44.459</t>
+  </si>
+  <si>
     <t xml:space="preserve">OSEM (2D)</t>
   </si>
   <si>
@@ -88,6 +103,12 @@
     <t xml:space="preserve">0.876298 +/- 0.059196</t>
   </si>
   <si>
+    <t xml:space="preserve">49.960 +/- 73.618</t>
+  </si>
+  <si>
+    <t xml:space="preserve">41.276 +/- 57.065</t>
+  </si>
+  <si>
     <t xml:space="preserve">ACT</t>
   </si>
   <si>
@@ -106,6 +127,12 @@
     <t xml:space="preserve">0.870791 +/- 0.068606</t>
   </si>
   <si>
+    <t xml:space="preserve">50.848 +/- 77.452</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A</t>
+  </si>
+  <si>
     <t xml:space="preserve">Could train 200 more epochs</t>
   </si>
   <si>
@@ -121,6 +148,9 @@
     <t xml:space="preserve">0.867473 +/- 0.062447</t>
   </si>
   <si>
+    <t xml:space="preserve">B</t>
+  </si>
+  <si>
     <t xml:space="preserve">Could trai n200 more epochs</t>
   </si>
   <si>
@@ -130,12 +160,18 @@
     <t xml:space="preserve">0.883188 +/- 0.062850</t>
   </si>
   <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.899746 +/- 0.068969</t>
   </si>
   <si>
     <t xml:space="preserve">0.897186 +/- 0.059042</t>
   </si>
   <si>
+    <t xml:space="preserve">D</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sinogram</t>
   </si>
   <si>
@@ -145,7 +181,10 @@
     <t xml:space="preserve">0.903350 +/- 0.057515</t>
   </si>
   <si>
-    <t xml:space="preserve">FILL IN</t>
+    <t xml:space="preserve">39.636 +/- 58.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E</t>
   </si>
   <si>
     <t xml:space="preserve">Early stopping at 370 epochs resolved THREE hotspots</t>
@@ -154,6 +193,9 @@
     <t xml:space="preserve">288x218</t>
   </si>
   <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
     <t xml:space="preserve">288x180</t>
   </si>
   <si>
@@ -161,6 +203,9 @@
   </si>
   <si>
     <t xml:space="preserve">0.892577 +/- 0.063994</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
   </si>
   <si>
     <t xml:space="preserve">First time the 17 mm hot spot showed up for full training</t>
@@ -249,7 +294,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -278,6 +323,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -302,15 +351,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -503,477 +544,572 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P1048576"/>
+  <dimension ref="B1:U1048576"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12.92"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="6.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="6.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="20.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="18.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="2" width="9.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="2" width="10.24"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="14" min="14" style="3" width="8.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="11.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="10.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="6.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="6.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="21.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="18.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="2" width="9.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="2" width="10.25"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="15" min="15" style="3" width="8.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="3" width="18.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="3" width="16.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="3" width="11.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="10.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="11.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4"/>
       <c r="I1" s="4"/>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="4"/>
+      <c r="K1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="5"/>
       <c r="L1" s="5"/>
       <c r="M1" s="5"/>
-      <c r="N1" s="6"/>
-      <c r="P1" s="2"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="U1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="35.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
-      <c r="H2" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="H2" s="4"/>
       <c r="I2" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="J2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="J2" s="4" t="s">
         <v>11</v>
       </c>
+      <c r="K2" s="8" t="s">
+        <v>12</v>
+      </c>
       <c r="L2" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="Q2" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>15</v>
+      <c r="R2" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>17</v>
+      <c r="B3" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="L3" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M3" s="2" t="n">
         <v>0.913735</v>
       </c>
-      <c r="M3" s="3" t="n">
+      <c r="N3" s="3" t="n">
         <v>35.374</v>
       </c>
-      <c r="N3" s="3" t="n">
+      <c r="O3" s="3" t="n">
         <v>46.275</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="R3" s="3" t="n">
+        <v>59.466</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>20</v>
+      <c r="B4" s="1" t="s">
+        <v>24</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L4" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M4" s="11" t="n">
         <v>0.85964</v>
       </c>
-      <c r="M4" s="3" t="n">
+      <c r="N4" s="3" t="n">
         <v>21.007</v>
       </c>
-      <c r="N4" s="3" t="n">
+      <c r="O4" s="3" t="n">
         <v>30.645</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <v>84.584</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="1" t="n">
         <v>288</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="1" t="n">
+      <c r="D5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F5" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="1" t="n">
+      <c r="I5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I5" s="1" t="n">
+      <c r="J5" s="1" t="n">
         <v>600</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="K5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="L5" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M5" s="2" t="n">
         <v>0.793076</v>
       </c>
-      <c r="M5" s="3" t="n">
+      <c r="N5" s="3" t="n">
         <v>3.77</v>
       </c>
-      <c r="N5" s="3" t="n">
+      <c r="O5" s="3" t="n">
         <v>5.642</v>
       </c>
-      <c r="P5" s="1" t="s">
-        <v>28</v>
+      <c r="P5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>45.469</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>119.861</v>
+      </c>
+      <c r="S5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="1" t="n">
+      <c r="B6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="1" t="n">
         <v>288</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="D6" s="1" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="1" t="n">
+      <c r="I6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I6" s="1" t="n">
+      <c r="J6" s="1" t="n">
         <v>600</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="K6" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="L6" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M6" s="2" t="n">
         <v>0.831867</v>
       </c>
-      <c r="M6" s="3" t="n">
+      <c r="N6" s="3" t="n">
         <v>4.947</v>
       </c>
-      <c r="N6" s="3" t="n">
+      <c r="O6" s="3" t="n">
         <v>1.364</v>
       </c>
-      <c r="P6" s="1" t="s">
-        <v>33</v>
+      <c r="P6" s="3" t="n">
+        <v>52.781</v>
+      </c>
+      <c r="Q6" s="3" t="n">
+        <v>45.313</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>108.83</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="T6" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="1" t="n">
+      <c r="B7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="1" t="n">
         <v>288</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="1" t="n">
+      <c r="D7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F7" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="1" t="n">
+      <c r="I7" s="1" t="n">
         <v>0.3</v>
       </c>
-      <c r="I7" s="1" t="n">
+      <c r="J7" s="1" t="n">
         <v>800</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="K7" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="L7" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="M7" s="2" t="n">
         <v>0.825372</v>
       </c>
-      <c r="M7" s="3" t="n">
+      <c r="N7" s="3" t="n">
         <v>3.086</v>
       </c>
-      <c r="N7" s="3" t="n">
+      <c r="O7" s="3" t="n">
         <v>1.457</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>49.239</v>
+      </c>
+      <c r="Q7" s="3" t="n">
+        <v>45.602</v>
+      </c>
+      <c r="R7" s="3" t="n">
+        <v>111.389</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="1" t="n">
+      <c r="B8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="1" t="n">
         <v>288</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="D8" s="1" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H8" s="1" t="n">
+      <c r="I8" s="1" t="n">
         <v>0.3</v>
       </c>
-      <c r="I8" s="1" t="n">
+      <c r="J8" s="1" t="n">
         <v>800</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="K8" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="L8" s="2" t="n">
+      <c r="K8" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="L8" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="M8" s="2" t="n">
         <v>0.835666</v>
       </c>
-      <c r="M8" s="3" t="n">
+      <c r="N8" s="3" t="n">
         <v>4.56</v>
       </c>
-      <c r="N8" s="3" t="n">
+      <c r="O8" s="3" t="n">
         <v>0.197</v>
+      </c>
+      <c r="R8" s="3" t="n">
+        <v>103.829</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="1" t="n">
+      <c r="B9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="1" t="n">
         <v>288</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="D9" s="1" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="G9" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H9" s="1" t="n">
+      <c r="I9" s="1" t="n">
         <v>0.3</v>
       </c>
-      <c r="I9" s="1" t="n">
+      <c r="J9" s="1" t="n">
         <v>800</v>
       </c>
-      <c r="J9" s="1" t="s">
-        <v>39</v>
-      </c>
       <c r="K9" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="L9" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="M9" s="2" t="n">
         <v>0.878936</v>
       </c>
-      <c r="M9" s="2" t="n">
-        <v>14.327</v>
-      </c>
-      <c r="N9" s="3" t="n">
+      <c r="N9" s="2" t="n">
+        <v>14.326</v>
+      </c>
+      <c r="O9" s="3" t="n">
         <v>7.15</v>
+      </c>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>82.625</v>
+      </c>
+      <c r="S9" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I10" s="1" t="n">
+      <c r="J10" s="1" t="n">
         <v>370</v>
       </c>
-      <c r="J10" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="K10" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="L10" s="2" t="n">
+      <c r="K10" s="13"/>
+      <c r="L10" s="13"/>
+      <c r="M10" s="2" t="n">
         <v>0.816511</v>
       </c>
-      <c r="M10" s="2" t="n">
+      <c r="N10" s="2" t="n">
         <v>15.42</v>
       </c>
-      <c r="N10" s="3" t="n">
+      <c r="O10" s="3" t="n">
         <v>4.178</v>
       </c>
-      <c r="P10" s="0" t="s">
-        <v>42</v>
+      <c r="R10" s="3" t="n">
+        <v>108.347</v>
+      </c>
+      <c r="T10" s="1" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="12" t="n">
+      <c r="B11" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="13" t="n">
         <v>288</v>
       </c>
-      <c r="C11" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="F11" s="12" t="s">
+      <c r="D11" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="G11" s="12" t="s">
+      <c r="E11" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="H11" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="H11" s="12" t="n">
+      <c r="I11" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="I11" s="12" t="n">
+      <c r="J11" s="13" t="n">
         <v>800</v>
       </c>
-      <c r="J11" s="12"/>
-      <c r="K11" s="13"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="13"/>
+      <c r="S11" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="1" t="n">
+      <c r="B12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="1" t="n">
         <v>288</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="D12" s="1" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="G12" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H12" s="1" t="n">
+      <c r="I12" s="1" t="n">
         <v>0.3</v>
       </c>
-      <c r="I12" s="1" t="n">
+      <c r="J12" s="1" t="n">
         <v>800</v>
       </c>
-      <c r="J12" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="K12" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="L12" s="14" t="n">
+        <v>59</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="M12" s="14" t="n">
         <v>0.808252704995019</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="N12" s="9" t="n">
         <v>6.353</v>
       </c>
-      <c r="N12" s="15" t="n">
+      <c r="O12" s="10" t="n">
         <v>11.175</v>
       </c>
-      <c r="P12" s="0" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0"/>
-      <c r="B13" s="0"/>
-      <c r="C13" s="0"/>
-      <c r="D13" s="0"/>
-      <c r="E13" s="0"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="10"/>
+      <c r="R12" s="10" t="n">
+        <v>109.952</v>
+      </c>
+      <c r="S12" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="T12" s="1" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A1:A2"/>
+  <mergeCells count="9">
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="F1:F2"/>
     <mergeCell ref="G1:G2"/>
-    <mergeCell ref="J1:L1"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="P1:R1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Implemented modality dropout scheduling
</commit_message>
<xml_diff>
--- a/project/network_performance.xlsx
+++ b/project/network_performance.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="67">
   <si>
     <t xml:space="preserve">Recon Type</t>
   </si>
@@ -181,16 +181,28 @@
     <t xml:space="preserve">0.903350 +/- 0.057515</t>
   </si>
   <si>
-    <t xml:space="preserve">39.636 +/- 58.000</t>
-  </si>
-  <si>
     <t xml:space="preserve">E</t>
   </si>
   <si>
+    <t xml:space="preserve">E (2)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Early stopping at 370 epochs resolved THREE hotspots</t>
   </si>
   <si>
     <t xml:space="preserve">288x218</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.922538 +/- 0.052700</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.900718 +/- 0.060376</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34.792 +/- 52.729</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40.399 +/- 59.270</t>
   </si>
   <si>
     <t xml:space="preserve">F</t>
@@ -557,7 +569,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="6.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="6.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="21.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="18.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="20.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="2" width="9.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="2" width="10.25"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="15" min="15" style="3" width="8.45"/>
@@ -755,9 +767,6 @@
       <c r="P5" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="Q5" s="3" t="n">
-        <v>45.469</v>
-      </c>
       <c r="R5" s="3" t="n">
         <v>119.861</v>
       </c>
@@ -811,12 +820,6 @@
       <c r="O6" s="3" t="n">
         <v>1.364</v>
       </c>
-      <c r="P6" s="3" t="n">
-        <v>52.781</v>
-      </c>
-      <c r="Q6" s="3" t="n">
-        <v>45.313</v>
-      </c>
       <c r="R6" s="3" t="n">
         <v>108.83</v>
       </c>
@@ -870,12 +873,6 @@
       <c r="O7" s="3" t="n">
         <v>1.457</v>
       </c>
-      <c r="P7" s="3" t="n">
-        <v>49.239</v>
-      </c>
-      <c r="Q7" s="3" t="n">
-        <v>45.602</v>
-      </c>
       <c r="R7" s="3" t="n">
         <v>111.389</v>
       </c>
@@ -970,21 +967,19 @@
       <c r="M9" s="2" t="n">
         <v>0.878936</v>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="N9" s="3" t="n">
         <v>14.326</v>
       </c>
       <c r="O9" s="3" t="n">
         <v>7.15</v>
       </c>
       <c r="P9" s="2"/>
-      <c r="Q9" s="2" t="s">
-        <v>53</v>
-      </c>
+      <c r="Q9" s="2"/>
       <c r="R9" s="2" t="n">
         <v>82.625</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -996,7 +991,7 @@
       <c r="M10" s="2" t="n">
         <v>0.816511</v>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="N10" s="3" t="n">
         <v>15.42</v>
       </c>
       <c r="O10" s="3" t="n">
@@ -1004,6 +999,9 @@
       </c>
       <c r="R10" s="3" t="n">
         <v>108.347</v>
+      </c>
+      <c r="S10" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="T10" s="1" t="s">
         <v>55</v>
@@ -1013,34 +1011,56 @@
       <c r="B11" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="12" t="n">
         <v>288</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="G11" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="I11" s="13" t="n">
+      <c r="I11" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="J11" s="13" t="n">
         <v>800</v>
       </c>
-      <c r="K11" s="12"/>
-      <c r="L11" s="13"/>
+      <c r="K11" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="L11" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>0.815321</v>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>6.142</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>3.345</v>
+      </c>
+      <c r="P11" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="R11" s="3" t="n">
+        <v>119.885</v>
+      </c>
       <c r="S11" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1057,7 +1077,7 @@
         <v>39</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>50</v>
@@ -1072,15 +1092,15 @@
         <v>800</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="M12" s="14" t="n">
         <v>0.808252704995019</v>
       </c>
-      <c r="N12" s="9" t="n">
+      <c r="N12" s="10" t="n">
         <v>6.353</v>
       </c>
       <c r="O12" s="10" t="n">
@@ -1092,11 +1112,17 @@
         <v>109.952</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>62</v>
-      </c>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N13" s="3"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N14" s="3"/>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>

</xml_diff>

<commit_message>
just checking batch files work
</commit_message>
<xml_diff>
--- a/project/network_performance.xlsx
+++ b/project/network_performance.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="88">
   <si>
     <t xml:space="preserve">Recon Type</t>
   </si>
@@ -43,9 +43,6 @@
     <t xml:space="preserve">Tuned For</t>
   </si>
   <si>
-    <t xml:space="preserve">Enforce Settings</t>
-  </si>
-  <si>
     <t xml:space="preserve">SSIM</t>
   </si>
   <si>
@@ -64,10 +61,7 @@
     <t xml:space="preserve"># epochs</t>
   </si>
   <si>
-    <t xml:space="preserve">Train Config</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Search Config</t>
+    <t xml:space="preserve">Enforced</t>
   </si>
   <si>
     <t xml:space="preserve">training set</t>
@@ -175,9 +169,6 @@
     <t xml:space="preserve">B</t>
   </si>
   <si>
-    <t xml:space="preserve">Could trai n200 more epochs</t>
-  </si>
-  <si>
     <t xml:space="preserve">0.889177 +/- 0.070444</t>
   </si>
   <si>
@@ -287,6 +278,9 @@
   </si>
   <si>
     <t xml:space="preserve">Fresh tuning with dropout=True enforced</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I</t>
   </si>
   <si>
     <t xml:space="preserve">Here, I started reducing fill choices to [0,1]</t>
@@ -727,7 +721,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:W1048576"/>
+  <dimension ref="A1:V1048576"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.38"/>
@@ -740,18 +734,18 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="6.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="6.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="7.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="8.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="21.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="20.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="2" width="9.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="2" width="10.25"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="17" min="17" style="3" width="8.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="3" width="18.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="3" width="16.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="3" width="11.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="10.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="11.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="8.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="21.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="20.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="2" width="9.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="2" width="10.25"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16" min="16" style="3" width="8.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="3" width="18.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="3" width="16.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="3" width="11.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="10.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="11.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -778,30 +772,27 @@
       </c>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="5"/>
+      <c r="L1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="5"/>
-      <c r="M1" s="6" t="s">
-        <v>8</v>
-      </c>
+      <c r="M1" s="6"/>
       <c r="N1" s="6"/>
       <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="8" t="s">
+      <c r="P1" s="7"/>
+      <c r="Q1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="R1" s="8"/>
+      <c r="S1" s="8"/>
+      <c r="T1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="S1" s="8"/>
-      <c r="T1" s="8"/>
-      <c r="U1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="W1" s="2"/>
+      <c r="V1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="35.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -811,48 +802,45 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="9" t="s">
+      <c r="N2" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="9" t="s">
+      <c r="O2" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="10" t="s">
+      <c r="P2" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="10" t="s">
+      <c r="Q2" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="U2" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="R2" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="S2" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="T2" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
@@ -863,36 +851,35 @@
       <c r="I3" s="13"/>
       <c r="J3" s="13"/>
       <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
+      <c r="L3" s="14" t="s">
+        <v>22</v>
+      </c>
       <c r="M3" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="13" t="n">
+        <v>0.913735</v>
+      </c>
+      <c r="O3" s="15" t="n">
+        <v>35.374</v>
+      </c>
+      <c r="P3" s="15" t="n">
+        <v>46.275</v>
+      </c>
+      <c r="Q3" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="N3" s="14" t="s">
+      <c r="R3" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="O3" s="13" t="n">
-        <v>0.913735</v>
-      </c>
-      <c r="P3" s="15" t="n">
-        <v>35.374</v>
-      </c>
-      <c r="Q3" s="15" t="n">
-        <v>46.275</v>
-      </c>
-      <c r="R3" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="S3" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="T3" s="17" t="n">
+      <c r="S3" s="17" t="n">
         <v>59.466</v>
       </c>
-      <c r="U3" s="2"/>
+      <c r="T3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C4" s="19"/>
       <c r="D4" s="19"/>
@@ -903,57 +890,56 @@
       <c r="I4" s="19"/>
       <c r="J4" s="19"/>
       <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
+      <c r="L4" s="19" t="s">
+        <v>27</v>
+      </c>
       <c r="M4" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="N4" s="20" t="n">
+        <v>0.85964</v>
+      </c>
+      <c r="O4" s="21" t="n">
+        <v>21.007</v>
+      </c>
+      <c r="P4" s="21" t="n">
+        <v>30.645</v>
+      </c>
+      <c r="Q4" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="N4" s="19" t="s">
+      <c r="R4" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="O4" s="20" t="n">
-        <v>0.85964</v>
-      </c>
-      <c r="P4" s="21" t="n">
-        <v>21.007</v>
-      </c>
-      <c r="Q4" s="21" t="n">
-        <v>30.645</v>
-      </c>
-      <c r="R4" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="S4" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="T4" s="22" t="n">
+      <c r="S4" s="22" t="n">
         <v>84.584</v>
       </c>
-      <c r="U4" s="2"/>
+      <c r="T4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>288</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>2</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>1</v>
@@ -962,62 +948,61 @@
         <v>600</v>
       </c>
       <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
+      <c r="L5" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="M5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>0.793076</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>5.642</v>
+      </c>
+      <c r="Q5" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="R5" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="O5" s="2" t="n">
-        <v>0.793076</v>
-      </c>
-      <c r="P5" s="3" t="n">
-        <v>3.77</v>
-      </c>
-      <c r="Q5" s="3" t="n">
-        <v>5.642</v>
-      </c>
-      <c r="R5" s="3" t="s">
+      <c r="S5" s="3" t="n">
+        <v>119.861</v>
+      </c>
+      <c r="T5" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="S5" s="3" t="s">
+      <c r="U5" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="T5" s="3" t="n">
-        <v>119.861</v>
-      </c>
-      <c r="U5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="V5" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>288</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>1</v>
@@ -1026,36 +1011,35 @@
         <v>600</v>
       </c>
       <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
+      <c r="L6" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="M6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>0.831867</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>4.947</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>1.364</v>
+      </c>
+      <c r="Q6" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="N6" s="2" t="s">
+      <c r="R6" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="O6" s="2" t="n">
-        <v>0.831867</v>
-      </c>
-      <c r="P6" s="3" t="n">
-        <v>4.947</v>
-      </c>
-      <c r="Q6" s="3" t="n">
-        <v>1.364</v>
-      </c>
-      <c r="R6" s="3" t="s">
+      <c r="S6" s="3" t="n">
+        <v>108.83</v>
+      </c>
+      <c r="T6" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="S6" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="T6" s="3" t="n">
-        <v>108.83</v>
-      </c>
-      <c r="U6" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="V6" s="1" t="s">
-        <v>51</v>
+      <c r="U6" s="1" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1063,25 +1047,25 @@
         <v>2</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>288</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>2</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I7" s="2" t="n">
         <v>0.3</v>
@@ -1090,33 +1074,32 @@
         <v>800</v>
       </c>
       <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
+      <c r="L7" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="M7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>0.825372</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>3.086</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>1.457</v>
+      </c>
+      <c r="Q7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="R7" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="S7" s="3" t="n">
+        <v>111.389</v>
+      </c>
+      <c r="T7" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="O7" s="2" t="n">
-        <v>0.825372</v>
-      </c>
-      <c r="P7" s="3" t="n">
-        <v>3.086</v>
-      </c>
-      <c r="Q7" s="3" t="n">
-        <v>1.457</v>
-      </c>
-      <c r="R7" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="S7" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="T7" s="3" t="n">
-        <v>111.389</v>
-      </c>
-      <c r="U7" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1124,25 +1107,25 @@
         <v>2</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>288</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I8" s="2" t="n">
         <v>0.3</v>
@@ -1151,33 +1134,32 @@
         <v>800</v>
       </c>
       <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2" t="s">
+      <c r="L8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="M8" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>0.835666</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="Q8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="R8" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="N8" s="9" t="s">
+      <c r="S8" s="3" t="n">
+        <v>103.829</v>
+      </c>
+      <c r="T8" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>0.835666</v>
-      </c>
-      <c r="P8" s="3" t="n">
-        <v>4.56</v>
-      </c>
-      <c r="Q8" s="3" t="n">
-        <v>0.197</v>
-      </c>
-      <c r="R8" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="S8" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="T8" s="3" t="n">
-        <v>103.829</v>
-      </c>
-      <c r="U8" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1185,25 +1167,25 @@
         <v>5</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C9" s="2" t="n">
         <v>288</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I9" s="2" t="n">
         <v>0.3</v>
@@ -1212,33 +1194,32 @@
         <v>800</v>
       </c>
       <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2" t="s">
+      <c r="L9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="M9" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>0.878936</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>14.326</v>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="Q9" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="R9" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="N9" s="23" t="s">
+      <c r="S9" s="2" t="n">
+        <v>82.625</v>
+      </c>
+      <c r="T9" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="O9" s="2" t="n">
-        <v>0.878936</v>
-      </c>
-      <c r="P9" s="3" t="n">
-        <v>14.326</v>
-      </c>
-      <c r="Q9" s="3" t="n">
-        <v>7.15</v>
-      </c>
-      <c r="R9" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="S9" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="T9" s="2" t="n">
-        <v>82.625</v>
-      </c>
-      <c r="U9" s="2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1254,53 +1235,52 @@
         <v>370</v>
       </c>
       <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
+      <c r="L10" s="9"/>
       <c r="M10" s="9"/>
-      <c r="N10" s="9"/>
-      <c r="O10" s="2" t="n">
+      <c r="N10" s="2" t="n">
         <v>0.816511</v>
       </c>
+      <c r="O10" s="3" t="n">
+        <v>15.42</v>
+      </c>
       <c r="P10" s="3" t="n">
-        <v>15.42</v>
-      </c>
-      <c r="Q10" s="3" t="n">
         <v>4.178</v>
       </c>
-      <c r="R10" s="2"/>
-      <c r="T10" s="3" t="n">
+      <c r="Q10" s="2"/>
+      <c r="S10" s="3" t="n">
         <v>108.347</v>
       </c>
-      <c r="U10" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="V10" s="1" t="s">
-        <v>69</v>
+      <c r="T10" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="U10" s="1" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C11" s="9" t="n">
         <v>288</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I11" s="9" t="n">
         <v>0.3</v>
@@ -1309,59 +1289,58 @@
         <v>800</v>
       </c>
       <c r="K11" s="23"/>
-      <c r="L11" s="23"/>
-      <c r="M11" s="23" t="s">
+      <c r="L11" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="M11" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>0.815321</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>6.142</v>
+      </c>
+      <c r="P11" s="3" t="n">
+        <v>3.345</v>
+      </c>
+      <c r="Q11" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="R11" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N11" s="9" t="s">
+      <c r="S11" s="3" t="n">
+        <v>119.885</v>
+      </c>
+      <c r="T11" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="O11" s="2" t="n">
-        <v>0.815321</v>
-      </c>
-      <c r="P11" s="3" t="n">
-        <v>6.142</v>
-      </c>
-      <c r="Q11" s="3" t="n">
-        <v>3.345</v>
-      </c>
-      <c r="R11" s="24" t="s">
-        <v>74</v>
-      </c>
-      <c r="S11" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="T11" s="3" t="n">
-        <v>119.885</v>
-      </c>
-      <c r="U11" s="2" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>288</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I12" s="2" t="n">
         <v>0.3</v>
@@ -1370,62 +1349,61 @@
         <v>800</v>
       </c>
       <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
+      <c r="L12" s="2" t="s">
+        <v>75</v>
+      </c>
       <c r="M12" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="N12" s="10" t="n">
+        <v>0.808252704995019</v>
+      </c>
+      <c r="O12" s="11" t="n">
+        <v>6.353</v>
+      </c>
+      <c r="P12" s="11" t="n">
+        <v>11.175</v>
+      </c>
+      <c r="Q12" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="R12" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="N12" s="2" t="s">
+      <c r="S12" s="11" t="n">
+        <v>109.952</v>
+      </c>
+      <c r="T12" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="O12" s="10" t="n">
-        <v>0.808252704995019</v>
-      </c>
-      <c r="P12" s="11" t="n">
-        <v>6.353</v>
-      </c>
-      <c r="Q12" s="11" t="n">
-        <v>11.175</v>
-      </c>
-      <c r="R12" s="11" t="s">
+      <c r="U12" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="S12" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="T12" s="11" t="n">
-        <v>109.952</v>
-      </c>
-      <c r="U12" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="V12" s="1" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C13" s="2" t="n">
         <v>288</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I13" s="2" t="n">
         <v>0.3</v>
@@ -1433,39 +1411,38 @@
       <c r="J13" s="2" t="n">
         <v>165</v>
       </c>
-      <c r="K13" s="2"/>
+      <c r="K13" s="2" t="s">
+        <v>82</v>
+      </c>
       <c r="L13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="R13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="S13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="T13" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="U13" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="O13" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="P13" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="Q13" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="R13" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="S13" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="T13" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="U13" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="V13" s="1" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1473,25 +1450,40 @@
         <v>1</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C14" s="2" t="n">
         <v>320</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
+      <c r="D14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>800</v>
+      </c>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="U14" s="2"/>
-      <c r="V14" s="1" t="s">
-        <v>89</v>
+      <c r="T14" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="U14" s="1" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1507,8 +1499,7 @@
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="U15" s="2"/>
+      <c r="T15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="2"/>
@@ -1523,8 +1514,7 @@
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="U16" s="2"/>
+      <c r="T16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="2"/>
@@ -1539,14 +1529,13 @@
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="U17" s="2"/>
+      <c r="T17" s="2"/>
     </row>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="9">
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
@@ -1554,9 +1543,8 @@
     <mergeCell ref="F1:F2"/>
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="H1:H2"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="R1:T1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="Q1:S1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Before making big changes to allow 'None' types in all fields.
</commit_message>
<xml_diff>
--- a/project/network_performance.xlsx
+++ b/project/network_performance.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="96">
   <si>
     <t xml:space="preserve">Recon Type</t>
   </si>
@@ -277,13 +277,37 @@
     <t xml:space="preserve">H</t>
   </si>
   <si>
-    <t xml:space="preserve">Fresh tuning with dropout=True enforced</t>
+    <t xml:space="preserve">Fresh tuning with dropout=True enforced. All networks after this set dropout=False</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.926144 +/- 0.053757</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.910757 +/- 0.059141</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34.362 +/- 53.834</t>
+  </si>
+  <si>
+    <t xml:space="preserve">37.709 +/- 58.653</t>
   </si>
   <si>
     <t xml:space="preserve">I</t>
   </si>
   <si>
     <t xml:space="preserve">Here, I started reducing fill choices to [0,1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fill=1, no skips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">need to train</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tuning showed slower learning but I haven’t trained</t>
   </si>
 </sst>
 </file>
@@ -431,7 +455,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -526,6 +550,14 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -734,7 +766,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="6.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="6.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="8.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="12.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="21.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="20.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="2" width="9.67"/>
@@ -745,7 +777,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="3" width="11.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="10.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="11.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1197,7 +1229,7 @@
       <c r="L9" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="M9" s="23" t="s">
+      <c r="M9" s="9" t="s">
         <v>61</v>
       </c>
       <c r="N9" s="2" t="n">
@@ -1285,11 +1317,11 @@
       <c r="I11" s="9" t="n">
         <v>0.3</v>
       </c>
-      <c r="J11" s="23" t="n">
+      <c r="J11" s="9" t="n">
         <v>800</v>
       </c>
       <c r="K11" s="23"/>
-      <c r="L11" s="23" t="s">
+      <c r="L11" s="9" t="s">
         <v>69</v>
       </c>
       <c r="M11" s="9" t="s">
@@ -1356,7 +1388,7 @@
         <v>76</v>
       </c>
       <c r="N12" s="10" t="n">
-        <v>0.808252704995019</v>
+        <v>0.808253</v>
       </c>
       <c r="O12" s="11" t="n">
         <v>6.353</v>
@@ -1474,32 +1506,90 @@
         <v>0.3</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>800</v>
+        <v>607</v>
       </c>
       <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
+      <c r="L14" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="M14" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>0.858335</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>5.076</v>
+      </c>
+      <c r="P14" s="3" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="Q14" s="26" t="s">
+        <v>88</v>
+      </c>
+      <c r="R14" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="S14" s="3" t="n">
+        <v>94.898</v>
+      </c>
       <c r="T14" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="U14" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="T15" s="2"/>
+      <c r="C15" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="S15" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="U15" s="1" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="2"/>

</xml_diff>